<commit_message>
feat: añade El millonario de la puerta de al lado
</commit_message>
<xml_diff>
--- a/content/Travel_More_Catalogo.xlsx
+++ b/content/Travel_More_Catalogo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\MisProyectos\travelandmore\content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF2B7BF7-B370-493B-B2B0-9D10BEC85CDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{635D4668-D4FC-4A83-8CCE-14A47595502A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_CONFIG" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="396">
   <si>
     <t>Travel &amp; More · Catálogo maestro</t>
   </si>
@@ -1204,6 +1204,27 @@
   </si>
   <si>
     <t>Me encanta el café de especialidad preparado con filtro. Podemos tener una buena cafetera espresso en casa, pero para mí el café filtrado tiene algo especial. Prepararlo poco a poco, ver cómo se extrae y poder apreciar con más claridad los aromas y matices del grano forma parte de la experiencia. Este portafiltros de porcelana es sencillo, bonito y cumple perfectamente: café, filtro de papel, agua y unos minutos para disfrutar del proceso. Para mí, como el café de filtro no hay nada :)</t>
+  </si>
+  <si>
+    <t>el-millonario-de-la-puerta-de-al-lado</t>
+  </si>
+  <si>
+    <t>assets/img/books/el-millonario-de-la-puerta-de-al-lado.jpg</t>
+  </si>
+  <si>
+    <t>El millonario de la puerta de al lado</t>
+  </si>
+  <si>
+    <t>Thomas J. Stanley, William D. Danko</t>
+  </si>
+  <si>
+    <t>Leyendo</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B01eV45RU</t>
+  </si>
+  <si>
+    <t>Un estudio sobre los hábitos y decisiones de personas que han conseguido acumular patrimonio sin llevar necesariamente un estilo de vida ostentoso. Thomas J. Stanley y William D. Danko analizan cómo viven, ahorran, consumen e invierten muchos millonarios, cuestionando la imagen tradicional que solemos asociar con la riqueza.</t>
   </si>
 </sst>
 </file>
@@ -7489,21 +7510,43 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
+    <row r="6" spans="1:14" ht="99">
+      <c r="A6" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>395</v>
+      </c>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
-      <c r="M6" s="4"/>
-      <c r="N6" s="4"/>
+      <c r="L6" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N6" s="4">
+        <v>5</v>
+      </c>
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="4"/>
@@ -9190,11 +9233,24 @@
     <hyperlink ref="L4" r:id="rId6" xr:uid="{00000000-0004-0000-0300-000005000000}"/>
     <hyperlink ref="K5" r:id="rId7" xr:uid="{00000000-0004-0000-0300-000006000000}"/>
     <hyperlink ref="L5" r:id="rId8" xr:uid="{00000000-0004-0000-0300-000007000000}"/>
+    <hyperlink ref="L6" r:id="rId9" xr:uid="{D7F5CD8C-95F6-45CF-A6CD-8ED50E6EEEA6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId9"/>
+    <tablePart r:id="rId10"/>
   </tableParts>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5B4E2C73-7564-48BC-9514-85A0837555B6}">
+          <x14:formula1>
+            <xm:f>'03_CATEGORIAS_LIBROS'!$B$2:$B$12</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2:E101</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 

</xml_diff>